<commit_message>
12 month historical price charts
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -493,19 +493,19 @@
         <v>131.31</v>
       </c>
       <c r="E2" t="n">
-        <v>167.52</v>
+        <v>165.17</v>
       </c>
       <c r="F2" t="n">
-        <v>4020.48</v>
+        <v>3964.08</v>
       </c>
       <c r="G2" t="n">
         <v>3151.44</v>
       </c>
       <c r="H2" t="n">
-        <v>869.04</v>
+        <v>812.64</v>
       </c>
       <c r="I2" t="n">
-        <v>27.58</v>
+        <v>25.79</v>
       </c>
     </row>
     <row r="3">
@@ -526,19 +526,19 @@
         <v>122.61</v>
       </c>
       <c r="E3" t="n">
-        <v>201.99</v>
+        <v>196.04</v>
       </c>
       <c r="F3" t="n">
-        <v>3231.84</v>
+        <v>3136.64</v>
       </c>
       <c r="G3" t="n">
         <v>1961.76</v>
       </c>
       <c r="H3" t="n">
-        <v>1270.08</v>
+        <v>1174.88</v>
       </c>
       <c r="I3" t="n">
-        <v>64.73999999999999</v>
+        <v>59.89</v>
       </c>
     </row>
     <row r="4">
@@ -559,19 +559,19 @@
         <v>744.67</v>
       </c>
       <c r="E4" t="n">
-        <v>1302.47</v>
+        <v>1253.96</v>
       </c>
       <c r="F4" t="n">
-        <v>6742.89</v>
+        <v>6491.75</v>
       </c>
       <c r="G4" t="n">
         <v>3855.16</v>
       </c>
       <c r="H4" t="n">
-        <v>2887.73</v>
+        <v>2636.59</v>
       </c>
       <c r="I4" t="n">
-        <v>74.91</v>
+        <v>68.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
complete portfolio dashboard - full automation
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,20 +456,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>52W High</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>52W Low</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Profit</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Return %</t>
         </is>
@@ -493,19 +503,25 @@
         <v>131.31</v>
       </c>
       <c r="E2" t="n">
-        <v>165.17</v>
+        <v>174.4</v>
       </c>
       <c r="F2" t="n">
-        <v>3964.08</v>
+        <v>212.19</v>
       </c>
       <c r="G2" t="n">
+        <v>86.62</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4185.6</v>
+      </c>
+      <c r="I2" t="n">
         <v>3151.44</v>
       </c>
-      <c r="H2" t="n">
-        <v>812.64</v>
-      </c>
-      <c r="I2" t="n">
-        <v>25.79</v>
+      <c r="J2" t="n">
+        <v>1034.16</v>
+      </c>
+      <c r="K2" t="n">
+        <v>32.82</v>
       </c>
     </row>
     <row r="3">
@@ -526,19 +542,25 @@
         <v>122.61</v>
       </c>
       <c r="E3" t="n">
-        <v>196.04</v>
+        <v>203.43</v>
       </c>
       <c r="F3" t="n">
-        <v>3136.64</v>
+        <v>267.08</v>
       </c>
       <c r="G3" t="n">
+        <v>76.48</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3254.88</v>
+      </c>
+      <c r="I3" t="n">
         <v>1961.76</v>
       </c>
-      <c r="H3" t="n">
-        <v>1174.88</v>
-      </c>
-      <c r="I3" t="n">
-        <v>59.89</v>
+      <c r="J3" t="n">
+        <v>1293.12</v>
+      </c>
+      <c r="K3" t="n">
+        <v>65.92</v>
       </c>
     </row>
     <row r="4">
@@ -559,19 +581,25 @@
         <v>744.67</v>
       </c>
       <c r="E4" t="n">
-        <v>1253.96</v>
+        <v>1320.83</v>
       </c>
       <c r="F4" t="n">
-        <v>6491.75</v>
+        <v>1547.22</v>
       </c>
       <c r="G4" t="n">
+        <v>578.51</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6837.94</v>
+      </c>
+      <c r="I4" t="n">
         <v>3855.16</v>
       </c>
-      <c r="H4" t="n">
-        <v>2636.59</v>
-      </c>
-      <c r="I4" t="n">
-        <v>68.39</v>
+      <c r="J4" t="n">
+        <v>2982.78</v>
+      </c>
+      <c r="K4" t="n">
+        <v>77.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>